<commit_message>
Set promotion window to 1 Jul - 31 Aug 2026 for all brands
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RBcJ9tq1t2zy8DPgHaL8X2
</commit_message>
<xml_diff>
--- a/Valeri_Pmax_Eight_Summer_Sales_2026.xlsx
+++ b/Valeri_Pmax_Eight_Summer_Sales_2026.xlsx
@@ -5369,7 +5369,7 @@
         </is>
       </c>
       <c r="DO94" s="1" t="n">
-        <v>46219</v>
+        <v>46204</v>
       </c>
       <c r="DP94" s="1" t="n">
         <v>46265</v>
@@ -5452,7 +5452,7 @@
         </is>
       </c>
       <c r="DO95" s="1" t="n">
-        <v>46219</v>
+        <v>46204</v>
       </c>
       <c r="DP95" s="1" t="n">
         <v>46265</v>
@@ -5535,7 +5535,7 @@
         </is>
       </c>
       <c r="DO96" s="1" t="n">
-        <v>46219</v>
+        <v>46204</v>
       </c>
       <c r="DP96" s="1" t="n">
         <v>46265</v>
@@ -5618,7 +5618,7 @@
         </is>
       </c>
       <c r="DO97" s="1" t="n">
-        <v>46219</v>
+        <v>46204</v>
       </c>
       <c r="DP97" s="1" t="n">
         <v>46265</v>
@@ -5701,7 +5701,7 @@
         </is>
       </c>
       <c r="DO98" s="1" t="n">
-        <v>46219</v>
+        <v>46204</v>
       </c>
       <c r="DP98" s="1" t="n">
         <v>46265</v>

</xml_diff>